<commit_message>
Update Laydown module 2 spreadsheet
</commit_message>
<xml_diff>
--- a/Laydown1_Module2.xlsx
+++ b/Laydown1_Module2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\material on laydown\outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA92E9FE-C683-4AC2-9CD1-34E92DE3A6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5A8BEE-12B9-4BC7-A368-55A98BBFD5DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="625" uniqueCount="149">
   <si>
     <t>Date</t>
   </si>
@@ -475,7 +475,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -755,7 +755,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="C3:J106"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="3" max="3" width="11.8984375" customWidth="1"/>
     <col min="4" max="4" width="11.19921875" customWidth="1"/>
@@ -765,7 +765,7 @@
     <col min="10" max="10" width="14.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:10">
       <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
@@ -782,7 +782,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:10">
       <c r="C4" s="4" t="s">
         <v>31</v>
       </c>
@@ -799,7 +799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:10">
       <c r="C5" s="4" t="s">
         <v>31</v>
       </c>
@@ -816,7 +816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:10">
       <c r="C6" s="4" t="s">
         <v>31</v>
       </c>
@@ -833,7 +833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:10">
       <c r="C7" s="4" t="s">
         <v>31</v>
       </c>
@@ -850,7 +850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:10">
       <c r="C8" s="4" t="s">
         <v>31</v>
       </c>
@@ -867,7 +867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:10">
       <c r="C9" s="4"/>
       <c r="D9" s="5"/>
       <c r="E9" s="4" t="s">
@@ -884,7 +884,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:10">
       <c r="C10" s="4"/>
       <c r="D10" s="5"/>
       <c r="E10" s="4" t="s">
@@ -897,7 +897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:10">
       <c r="C11" s="4"/>
       <c r="D11" s="5"/>
       <c r="E11" s="4" t="s">
@@ -910,7 +910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:10">
       <c r="C12" s="4" t="s">
         <v>5</v>
       </c>
@@ -927,7 +927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:10">
       <c r="C13" s="4"/>
       <c r="D13" s="5"/>
       <c r="E13" s="4" t="s">
@@ -940,7 +940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:10">
       <c r="C14" s="4" t="s">
         <v>5</v>
       </c>
@@ -957,7 +957,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:10">
       <c r="C15" s="4"/>
       <c r="D15" s="5"/>
       <c r="E15" s="4" t="s">
@@ -970,7 +970,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:10">
       <c r="C16" s="4"/>
       <c r="D16" s="5"/>
       <c r="E16" s="4" t="s">
@@ -983,7 +983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:7">
       <c r="C17" s="4"/>
       <c r="D17" s="5"/>
       <c r="E17" s="4" t="s">
@@ -996,7 +996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:7">
       <c r="C18" s="4" t="s">
         <v>5</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:7">
       <c r="C19" s="4"/>
       <c r="D19" s="5"/>
       <c r="E19" s="4" t="s">
@@ -1026,7 +1026,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:7">
       <c r="C20" s="4"/>
       <c r="D20" s="5"/>
       <c r="E20" s="4" t="s">
@@ -1039,7 +1039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:7">
       <c r="C21" s="4"/>
       <c r="D21" s="5"/>
       <c r="E21" s="4" t="s">
@@ -1052,7 +1052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:7">
       <c r="C22" s="4" t="s">
         <v>5</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:7">
       <c r="C23" s="4"/>
       <c r="D23" s="5"/>
       <c r="E23" s="4" t="s">
@@ -1082,7 +1082,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:7">
       <c r="C24" s="4" t="s">
         <v>36</v>
       </c>
@@ -1099,7 +1099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:7">
       <c r="C25" s="4" t="s">
         <v>31</v>
       </c>
@@ -1116,7 +1116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:7">
       <c r="C26" s="4"/>
       <c r="D26" s="5"/>
       <c r="E26" s="4" t="s">
@@ -1129,7 +1129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:7">
       <c r="C27" s="4"/>
       <c r="D27" s="5"/>
       <c r="E27" s="4" t="s">
@@ -1142,7 +1142,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:7">
       <c r="C28" s="4" t="s">
         <v>5</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:7">
       <c r="C29" s="4"/>
       <c r="D29" s="5"/>
       <c r="E29" s="4" t="s">
@@ -1172,7 +1172,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:7">
       <c r="C30" s="4" t="s">
         <v>5</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:7">
       <c r="C31" s="4"/>
       <c r="D31" s="5"/>
       <c r="E31" s="4" t="s">
@@ -1202,7 +1202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:7">
       <c r="C32" s="4"/>
       <c r="D32" s="5"/>
       <c r="E32" s="4" t="s">
@@ -1215,7 +1215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:7">
       <c r="C33" s="4"/>
       <c r="D33" s="5"/>
       <c r="E33" s="4" t="s">
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:7">
       <c r="C34" s="4" t="s">
         <v>36</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:7">
       <c r="C35" s="4" t="s">
         <v>31</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:7">
       <c r="C36" s="4"/>
       <c r="D36" s="5"/>
       <c r="E36" s="4" t="s">
@@ -1275,7 +1275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:7">
       <c r="C37" s="4" t="s">
         <v>31</v>
       </c>
@@ -1292,7 +1292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:7">
       <c r="C38" s="4"/>
       <c r="D38" s="5"/>
       <c r="E38" s="4" t="s">
@@ -1305,7 +1305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:7">
       <c r="C39" s="4" t="s">
         <v>36</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:7">
       <c r="C40" s="4" t="s">
         <v>5</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:7">
       <c r="C41" s="4"/>
       <c r="D41" s="5"/>
       <c r="E41" s="4" t="s">
@@ -1352,7 +1352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:7">
       <c r="C42" s="4"/>
       <c r="D42" s="5"/>
       <c r="E42" s="4" t="s">
@@ -1365,7 +1365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:7">
       <c r="C43" s="4"/>
       <c r="D43" s="5"/>
       <c r="E43" s="4" t="s">
@@ -1378,7 +1378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:7">
       <c r="C44" s="4"/>
       <c r="D44" s="5"/>
       <c r="E44" s="4" t="s">
@@ -1391,7 +1391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:7">
       <c r="C45" s="4"/>
       <c r="D45" s="5"/>
       <c r="E45" s="4" t="s">
@@ -1404,7 +1404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:7">
       <c r="C46" s="4"/>
       <c r="D46" s="5"/>
       <c r="E46" s="4" t="s">
@@ -1417,7 +1417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:7">
       <c r="C47" s="4" t="s">
         <v>36</v>
       </c>
@@ -1434,7 +1434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:7">
       <c r="C48" s="4"/>
       <c r="D48" s="5"/>
       <c r="E48" s="4" t="s">
@@ -1447,7 +1447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:7">
       <c r="C49" s="4" t="s">
         <v>36</v>
       </c>
@@ -1464,7 +1464,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:7">
       <c r="C50" s="4"/>
       <c r="D50" s="5"/>
       <c r="E50" s="4" t="s">
@@ -1477,7 +1477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:7">
       <c r="C51" s="4"/>
       <c r="D51" s="5"/>
       <c r="E51" s="4" t="s">
@@ -1490,7 +1490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:7">
       <c r="C52" s="4" t="s">
         <v>36</v>
       </c>
@@ -1507,7 +1507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:7">
       <c r="C53" s="4" t="s">
         <v>36</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:7">
       <c r="C54" s="4" t="s">
         <v>36</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:7">
       <c r="C55" s="4"/>
       <c r="D55" s="5"/>
       <c r="E55" s="4" t="s">
@@ -1554,7 +1554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="3:7">
       <c r="C56" s="4"/>
       <c r="D56" s="5"/>
       <c r="E56" s="4" t="s">
@@ -1567,7 +1567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="3:7">
       <c r="C57" s="4"/>
       <c r="D57" s="5"/>
       <c r="E57" s="4" t="s">
@@ -1580,7 +1580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="3:7">
       <c r="C58" s="4"/>
       <c r="D58" s="5"/>
       <c r="E58" s="4" t="s">
@@ -1593,7 +1593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="3:7">
       <c r="C59" s="4" t="s">
         <v>31</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="3:7">
       <c r="C60" s="4"/>
       <c r="D60" s="5"/>
       <c r="E60" s="4" t="s">
@@ -1623,7 +1623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="3:7">
       <c r="C61" s="4"/>
       <c r="D61" s="5"/>
       <c r="E61" s="4" t="s">
@@ -1636,7 +1636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="3:7">
       <c r="C62" s="4"/>
       <c r="D62" s="5"/>
       <c r="E62" s="4" t="s">
@@ -1649,7 +1649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="3:7">
       <c r="C63" s="4"/>
       <c r="D63" s="5"/>
       <c r="E63" s="4" t="s">
@@ -1662,7 +1662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="3:7">
       <c r="C64" s="4" t="s">
         <v>36</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:7">
       <c r="C65" s="4"/>
       <c r="D65" s="5"/>
       <c r="E65" s="4" t="s">
@@ -1692,7 +1692,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="3:7">
       <c r="C66" s="4"/>
       <c r="D66" s="5"/>
       <c r="E66" s="4" t="s">
@@ -1705,7 +1705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="3:7">
       <c r="C67" s="4"/>
       <c r="D67" s="5"/>
       <c r="E67" s="4" t="s">
@@ -1718,7 +1718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="3:7">
       <c r="C68" s="4"/>
       <c r="D68" s="5"/>
       <c r="E68" s="4" t="s">
@@ -1731,7 +1731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="3:7">
       <c r="C69" s="4"/>
       <c r="D69" s="5"/>
       <c r="E69" s="4" t="s">
@@ -1744,7 +1744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="3:7">
       <c r="C70" s="4"/>
       <c r="D70" s="5"/>
       <c r="E70" s="4" t="s">
@@ -1757,7 +1757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="3:7">
       <c r="C71" s="4"/>
       <c r="D71" s="5"/>
       <c r="E71" s="4" t="s">
@@ -1770,7 +1770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="3:7">
       <c r="C72" s="4" t="s">
         <v>36</v>
       </c>
@@ -1787,7 +1787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="3:7">
       <c r="C73" s="4" t="s">
         <v>36</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="3:7">
       <c r="C74" s="4"/>
       <c r="D74" s="5"/>
       <c r="E74" s="4" t="s">
@@ -1817,7 +1817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="3:7">
       <c r="C75" s="4"/>
       <c r="D75" s="5"/>
       <c r="E75" s="4" t="s">
@@ -1830,7 +1830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="3:7">
       <c r="C76" s="4"/>
       <c r="D76" s="5"/>
       <c r="E76" s="4" t="s">
@@ -1843,7 +1843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="3:7">
       <c r="C77" s="4"/>
       <c r="D77" s="5"/>
       <c r="E77" s="4" t="s">
@@ -1856,7 +1856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:7">
       <c r="C78" s="4"/>
       <c r="D78" s="5"/>
       <c r="E78" s="4" t="s">
@@ -1869,7 +1869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="3:7">
       <c r="C79" s="4"/>
       <c r="D79" s="5"/>
       <c r="E79" s="4" t="s">
@@ -1882,7 +1882,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="3:7">
       <c r="C80" s="4"/>
       <c r="D80" s="5"/>
       <c r="E80" s="4" t="s">
@@ -1895,7 +1895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="3:7">
       <c r="C81" s="4"/>
       <c r="D81" s="5"/>
       <c r="E81" s="4" t="s">
@@ -1908,7 +1908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="3:7">
       <c r="C82" s="4"/>
       <c r="D82" s="5"/>
       <c r="E82" s="4" t="s">
@@ -1921,7 +1921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:7">
       <c r="C83" s="4"/>
       <c r="D83" s="5"/>
       <c r="E83" s="4" t="s">
@@ -1934,7 +1934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="3:7">
       <c r="C84" s="4"/>
       <c r="D84" s="5"/>
       <c r="E84" s="4" t="s">
@@ -1947,7 +1947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="3:7">
       <c r="C85" s="4"/>
       <c r="D85" s="5"/>
       <c r="E85" s="4" t="s">
@@ -1960,7 +1960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="3:7">
       <c r="C86" s="4"/>
       <c r="D86" s="5"/>
       <c r="E86" s="4" t="s">
@@ -1973,7 +1973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="3:7">
       <c r="C87" s="4"/>
       <c r="D87" s="5"/>
       <c r="E87" s="4" t="s">
@@ -1986,7 +1986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="3:7">
       <c r="C88" s="4"/>
       <c r="D88" s="5"/>
       <c r="E88" s="4" t="s">
@@ -1999,7 +1999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="3:7">
       <c r="C89" s="4"/>
       <c r="D89" s="5"/>
       <c r="E89" s="4" t="s">
@@ -2012,7 +2012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="3:7">
       <c r="C90" s="4"/>
       <c r="D90" s="5"/>
       <c r="E90" s="4" t="s">
@@ -2025,7 +2025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="3:7">
       <c r="C91" s="4"/>
       <c r="D91" s="5"/>
       <c r="E91" s="4" t="s">
@@ -2038,7 +2038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="3:7">
       <c r="C92" s="4"/>
       <c r="D92" s="5"/>
       <c r="E92" s="4" t="s">
@@ -2051,7 +2051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="3:7">
       <c r="C93" s="4"/>
       <c r="D93" s="5"/>
       <c r="E93" s="4" t="s">
@@ -2064,7 +2064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="3:7">
       <c r="C94" s="4" t="s">
         <v>36</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="3:7">
       <c r="C95" s="4" t="s">
         <v>36</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="3:7">
       <c r="C96" s="4"/>
       <c r="D96" s="5"/>
       <c r="E96" s="4" t="s">
@@ -2111,7 +2111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="3:7">
       <c r="C97" s="4"/>
       <c r="D97" s="5"/>
       <c r="E97" s="4" t="s">
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="3:7">
       <c r="C98" s="4"/>
       <c r="D98" s="5"/>
       <c r="E98" s="4" t="s">
@@ -2137,7 +2137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="3:7">
       <c r="C99" s="4"/>
       <c r="D99" s="5"/>
       <c r="E99" s="4" t="s">
@@ -2150,7 +2150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="3:7">
       <c r="C100" s="4" t="s">
         <v>31</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="3:7">
       <c r="C101" s="4" t="s">
         <v>36</v>
       </c>
@@ -2184,7 +2184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="3:7">
       <c r="C102" s="4"/>
       <c r="D102" s="5"/>
       <c r="E102" s="4" t="s">
@@ -2197,7 +2197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="3:7">
       <c r="C103" s="4"/>
       <c r="D103" s="5"/>
       <c r="E103" s="4" t="s">
@@ -2210,7 +2210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="3:7">
       <c r="C104" s="4"/>
       <c r="D104" s="5"/>
       <c r="E104" s="4" t="s">
@@ -2223,7 +2223,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="3:7">
       <c r="C105" s="4"/>
       <c r="D105" s="5"/>
       <c r="E105" s="4" t="s">
@@ -2236,7 +2236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="3:7">
       <c r="C106" s="4"/>
       <c r="D106" s="5"/>
       <c r="E106" s="4" t="s">
@@ -2256,18 +2256,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="C3:J57"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="C3:M56"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="3" max="3" width="11.8984375" customWidth="1"/>
     <col min="4" max="4" width="11.19921875" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="16.19921875" customWidth="1"/>
     <col min="7" max="7" width="6.8984375" customWidth="1"/>
-    <col min="10" max="10" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="9.5" customWidth="1"/>
+    <col min="11" max="11" width="15.3984375" customWidth="1"/>
+    <col min="12" max="12" width="15.796875" customWidth="1"/>
+    <col min="13" max="13" width="7.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:13" ht="27.6">
       <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
@@ -2283,8 +2286,23 @@
       <c r="G3" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="I3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="3:13">
       <c r="C4" s="4"/>
       <c r="D4" s="5"/>
       <c r="E4" s="4" t="s">
@@ -2296,8 +2314,19 @@
       <c r="G4" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="I4" s="4"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="M4" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="3:13">
       <c r="C5" s="4"/>
       <c r="D5" s="5"/>
       <c r="E5" s="4" t="s">
@@ -2310,7 +2339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:13">
       <c r="C6" s="4"/>
       <c r="D6" s="5"/>
       <c r="E6" s="4" t="s">
@@ -2323,7 +2352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:13">
       <c r="C7" s="4"/>
       <c r="D7" s="5"/>
       <c r="E7" s="4" t="s">
@@ -2336,7 +2365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:13">
       <c r="C8" s="4"/>
       <c r="D8" s="5"/>
       <c r="E8" s="4" t="s">
@@ -2353,7 +2382,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="9" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:13">
       <c r="C9" s="4"/>
       <c r="D9" s="5"/>
       <c r="E9" s="4" t="s">
@@ -2366,7 +2395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:13">
       <c r="C10" s="4" t="s">
         <v>36</v>
       </c>
@@ -2383,7 +2412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:13">
       <c r="C11" s="4" t="s">
         <v>36</v>
       </c>
@@ -2400,7 +2429,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:13">
       <c r="C12" s="4"/>
       <c r="D12" s="5"/>
       <c r="E12" s="4" t="s">
@@ -2413,7 +2442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:13">
       <c r="C13" s="4"/>
       <c r="D13" s="5"/>
       <c r="E13" s="4" t="s">
@@ -2426,7 +2455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:13">
       <c r="C14" s="4"/>
       <c r="D14" s="5"/>
       <c r="E14" s="4" t="s">
@@ -2439,7 +2468,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:13">
       <c r="C15" s="4"/>
       <c r="D15" s="5"/>
       <c r="E15" s="4" t="s">
@@ -2452,7 +2481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:13">
       <c r="C16" s="4"/>
       <c r="D16" s="5"/>
       <c r="E16" s="4" t="s">
@@ -2465,7 +2494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:7">
       <c r="C17" s="4"/>
       <c r="D17" s="5"/>
       <c r="E17" s="4" t="s">
@@ -2478,7 +2507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:7">
       <c r="C18" s="4"/>
       <c r="D18" s="5"/>
       <c r="E18" s="4" t="s">
@@ -2491,7 +2520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:7">
       <c r="C19" s="4"/>
       <c r="D19" s="5"/>
       <c r="E19" s="4" t="s">
@@ -2504,7 +2533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:7">
       <c r="C20" s="4"/>
       <c r="D20" s="5"/>
       <c r="E20" s="4" t="s">
@@ -2517,7 +2546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:7">
       <c r="C21" s="4"/>
       <c r="D21" s="5"/>
       <c r="E21" s="4" t="s">
@@ -2530,7 +2559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:7">
       <c r="C22" s="4"/>
       <c r="D22" s="5"/>
       <c r="E22" s="4" t="s">
@@ -2543,7 +2572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:7">
       <c r="C23" s="4"/>
       <c r="D23" s="5"/>
       <c r="E23" s="4" t="s">
@@ -2556,7 +2585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:7">
       <c r="C24" s="4"/>
       <c r="D24" s="5"/>
       <c r="E24" s="4" t="s">
@@ -2569,7 +2598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:7">
       <c r="C25" s="4"/>
       <c r="D25" s="5"/>
       <c r="E25" s="4" t="s">
@@ -2582,7 +2611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:7">
       <c r="C26" s="4"/>
       <c r="D26" s="5"/>
       <c r="E26" s="4" t="s">
@@ -2595,7 +2624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:7">
       <c r="C27" s="4" t="s">
         <v>31</v>
       </c>
@@ -2612,7 +2641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:7">
       <c r="C28" s="4" t="s">
         <v>31</v>
       </c>
@@ -2629,7 +2658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:7">
       <c r="C29" s="4" t="s">
         <v>31</v>
       </c>
@@ -2646,7 +2675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:7">
       <c r="C30" s="4" t="s">
         <v>31</v>
       </c>
@@ -2663,7 +2692,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:7">
       <c r="C31" s="4" t="s">
         <v>31</v>
       </c>
@@ -2680,7 +2709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:7">
       <c r="C32" s="4"/>
       <c r="D32" s="5"/>
       <c r="E32" s="4" t="s">
@@ -2693,7 +2722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:7">
       <c r="C33" s="4"/>
       <c r="D33" s="5"/>
       <c r="E33" s="4" t="s">
@@ -2706,7 +2735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:7">
       <c r="C34" s="4" t="s">
         <v>36</v>
       </c>
@@ -2723,7 +2752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:7">
       <c r="C35" s="4" t="s">
         <v>36</v>
       </c>
@@ -2740,20 +2769,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:7">
       <c r="C36" s="4"/>
       <c r="D36" s="5"/>
       <c r="E36" s="4" t="s">
-        <v>86</v>
+        <v>7</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="G36" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:7">
       <c r="C37" s="4"/>
       <c r="D37" s="5"/>
       <c r="E37" s="4" t="s">
@@ -2766,20 +2795,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="4"/>
-      <c r="D38" s="5"/>
+    <row r="38" spans="3:7">
+      <c r="C38" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>37</v>
+      </c>
       <c r="E38" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="G38" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:7">
       <c r="C39" s="4" t="s">
         <v>36</v>
       </c>
@@ -2796,7 +2829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:7">
       <c r="C40" s="4" t="s">
         <v>36</v>
       </c>
@@ -2813,7 +2846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:7">
       <c r="C41" s="4" t="s">
         <v>36</v>
       </c>
@@ -2830,7 +2863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:7">
       <c r="C42" s="4" t="s">
         <v>36</v>
       </c>
@@ -2847,7 +2880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:7">
       <c r="C43" s="4" t="s">
         <v>36</v>
       </c>
@@ -2864,7 +2897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:7">
       <c r="C44" s="4" t="s">
         <v>36</v>
       </c>
@@ -2881,7 +2914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:7">
       <c r="C45" s="4" t="s">
         <v>36</v>
       </c>
@@ -2898,7 +2931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:7">
       <c r="C46" s="4" t="s">
         <v>36</v>
       </c>
@@ -2915,7 +2948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:7">
       <c r="C47" s="4" t="s">
         <v>36</v>
       </c>
@@ -2932,24 +2965,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C48" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>37</v>
-      </c>
+    <row r="48" spans="3:7">
+      <c r="C48" s="4"/>
+      <c r="D48" s="5"/>
       <c r="E48" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="G48" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:7">
       <c r="C49" s="4"/>
       <c r="D49" s="5"/>
       <c r="E49" s="4" t="s">
@@ -2962,20 +2991,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C50" s="4"/>
-      <c r="D50" s="5"/>
+    <row r="50" spans="3:7">
+      <c r="C50" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>32</v>
+      </c>
       <c r="E50" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="G50" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:7">
       <c r="C51" s="4" t="s">
         <v>31</v>
       </c>
@@ -2992,7 +3025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:7">
       <c r="C52" s="4" t="s">
         <v>31</v>
       </c>
@@ -3009,24 +3042,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:7">
       <c r="C53" s="4" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E53" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G53" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:7">
       <c r="C54" s="4" t="s">
         <v>36</v>
       </c>
@@ -3043,24 +3076,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:7">
       <c r="C55" s="4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E55" s="4" t="s">
         <v>7</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="G55" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="3:7">
       <c r="C56" s="4" t="s">
         <v>31</v>
       </c>
@@ -3074,23 +3107,6 @@
         <v>88</v>
       </c>
       <c r="G56" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D57" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E57" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F57" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="G57" s="5">
         <v>1</v>
       </c>
     </row>
@@ -3102,7 +3118,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="C3:J66"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="3" max="3" width="11.8984375" customWidth="1"/>
     <col min="4" max="4" width="11.19921875" customWidth="1"/>
@@ -3112,7 +3128,7 @@
     <col min="10" max="10" width="14.09765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:10">
       <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
@@ -3129,7 +3145,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:10">
       <c r="C4" s="4"/>
       <c r="D4" s="5"/>
       <c r="E4" s="4" t="s">
@@ -3142,7 +3158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:10">
       <c r="C5" s="4"/>
       <c r="D5" s="5"/>
       <c r="E5" s="4" t="s">
@@ -3155,7 +3171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:10">
       <c r="C6" s="4"/>
       <c r="D6" s="5"/>
       <c r="E6" s="4" t="s">
@@ -3168,7 +3184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:10">
       <c r="C7" s="4"/>
       <c r="D7" s="5"/>
       <c r="E7" s="4" t="s">
@@ -3185,7 +3201,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="8" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:10">
       <c r="C8" s="4" t="s">
         <v>120</v>
       </c>
@@ -3202,7 +3218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:10">
       <c r="C9" s="4" t="s">
         <v>120</v>
       </c>
@@ -3219,7 +3235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:10">
       <c r="C10" s="4" t="s">
         <v>120</v>
       </c>
@@ -3236,7 +3252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:10">
       <c r="C11" s="4" t="s">
         <v>120</v>
       </c>
@@ -3253,7 +3269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:10">
       <c r="C12" s="4"/>
       <c r="D12" s="5"/>
       <c r="E12" s="4" t="s">
@@ -3266,7 +3282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:10">
       <c r="C13" s="4" t="s">
         <v>120</v>
       </c>
@@ -3283,7 +3299,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:10">
       <c r="C14" s="4" t="s">
         <v>120</v>
       </c>
@@ -3300,7 +3316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:10">
       <c r="C15" s="4" t="s">
         <v>120</v>
       </c>
@@ -3317,7 +3333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="3:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:10">
       <c r="C16" s="4" t="s">
         <v>120</v>
       </c>
@@ -3334,7 +3350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:7">
       <c r="C17" s="4" t="s">
         <v>36</v>
       </c>
@@ -3351,7 +3367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:7">
       <c r="C18" s="4" t="s">
         <v>36</v>
       </c>
@@ -3368,7 +3384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:7">
       <c r="C19" s="4" t="s">
         <v>36</v>
       </c>
@@ -3385,7 +3401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:7">
       <c r="C20" s="4" t="s">
         <v>36</v>
       </c>
@@ -3402,7 +3418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:7">
       <c r="C21" s="4" t="s">
         <v>36</v>
       </c>
@@ -3419,7 +3435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:7">
       <c r="C22" s="4" t="s">
         <v>31</v>
       </c>
@@ -3436,7 +3452,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:7">
       <c r="C23" s="4"/>
       <c r="D23" s="5"/>
       <c r="E23" s="4" t="s">
@@ -3449,7 +3465,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:7">
       <c r="C24" s="4"/>
       <c r="D24" s="5"/>
       <c r="E24" s="4" t="s">
@@ -3462,7 +3478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:7">
       <c r="C25" s="4"/>
       <c r="D25" s="5"/>
       <c r="E25" s="4" t="s">
@@ -3475,7 +3491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:7">
       <c r="C26" s="4"/>
       <c r="D26" s="5"/>
       <c r="E26" s="4" t="s">
@@ -3488,7 +3504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:7">
       <c r="C27" s="4" t="s">
         <v>36</v>
       </c>
@@ -3505,7 +3521,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:7">
       <c r="C28" s="4" t="s">
         <v>120</v>
       </c>
@@ -3522,7 +3538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:7">
       <c r="C29" s="4"/>
       <c r="D29" s="5"/>
       <c r="E29" s="4" t="s">
@@ -3535,7 +3551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:7">
       <c r="C30" s="4"/>
       <c r="D30" s="5"/>
       <c r="E30" s="4" t="s">
@@ -3548,7 +3564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:7">
       <c r="C31" s="4"/>
       <c r="D31" s="5"/>
       <c r="E31" s="4" t="s">
@@ -3561,7 +3577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:7">
       <c r="C32" s="4"/>
       <c r="D32" s="5"/>
       <c r="E32" s="4" t="s">
@@ -3574,7 +3590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:7">
       <c r="C33" s="4" t="s">
         <v>120</v>
       </c>
@@ -3591,7 +3607,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:7">
       <c r="C34" s="4"/>
       <c r="D34" s="5"/>
       <c r="E34" s="4" t="s">
@@ -3604,7 +3620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:7">
       <c r="C35" s="4"/>
       <c r="D35" s="5"/>
       <c r="E35" s="4" t="s">
@@ -3617,7 +3633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:7">
       <c r="C36" s="4"/>
       <c r="D36" s="5"/>
       <c r="E36" s="4" t="s">
@@ -3630,7 +3646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:7">
       <c r="C37" s="4"/>
       <c r="D37" s="5"/>
       <c r="E37" s="4" t="s">
@@ -3643,7 +3659,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:7">
       <c r="C38" s="4"/>
       <c r="D38" s="5"/>
       <c r="E38" s="4" t="s">
@@ -3656,7 +3672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:7">
       <c r="C39" s="4"/>
       <c r="D39" s="5"/>
       <c r="E39" s="4" t="s">
@@ -3669,7 +3685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:7">
       <c r="C40" s="4"/>
       <c r="D40" s="5"/>
       <c r="E40" s="4" t="s">
@@ -3682,7 +3698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:7">
       <c r="C41" s="4"/>
       <c r="D41" s="5"/>
       <c r="E41" s="4" t="s">
@@ -3695,7 +3711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:7">
       <c r="C42" s="4"/>
       <c r="D42" s="5"/>
       <c r="E42" s="4" t="s">
@@ -3708,7 +3724,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:7">
       <c r="C43" s="4"/>
       <c r="D43" s="5"/>
       <c r="E43" s="4" t="s">
@@ -3721,7 +3737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:7">
       <c r="C44" s="4"/>
       <c r="D44" s="5"/>
       <c r="E44" s="4" t="s">
@@ -3734,7 +3750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:7">
       <c r="C45" s="4" t="s">
         <v>120</v>
       </c>
@@ -3751,7 +3767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:7">
       <c r="C46" s="4" t="s">
         <v>120</v>
       </c>
@@ -3768,7 +3784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:7">
       <c r="C47" s="4" t="s">
         <v>120</v>
       </c>
@@ -3785,7 +3801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:7">
       <c r="C48" s="4"/>
       <c r="D48" s="5"/>
       <c r="E48" s="4" t="s">
@@ -3798,7 +3814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:7">
       <c r="C49" s="4"/>
       <c r="D49" s="5"/>
       <c r="E49" s="4" t="s">
@@ -3811,7 +3827,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:7">
       <c r="C50" s="4"/>
       <c r="D50" s="5"/>
       <c r="E50" s="4" t="s">
@@ -3824,7 +3840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:7">
       <c r="C51" s="4"/>
       <c r="D51" s="5"/>
       <c r="E51" s="4" t="s">
@@ -3837,7 +3853,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:7">
       <c r="C52" s="4"/>
       <c r="D52" s="5"/>
       <c r="E52" s="4" t="s">
@@ -3850,7 +3866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:7">
       <c r="C53" s="4"/>
       <c r="D53" s="5"/>
       <c r="E53" s="4" t="s">
@@ -3863,7 +3879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:7">
       <c r="C54" s="4" t="s">
         <v>120</v>
       </c>
@@ -3880,7 +3896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:7">
       <c r="C55" s="4" t="s">
         <v>120</v>
       </c>
@@ -3897,7 +3913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="3:7">
       <c r="C56" s="4" t="s">
         <v>120</v>
       </c>
@@ -3914,7 +3930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="3:7">
       <c r="C57" s="4" t="s">
         <v>120</v>
       </c>
@@ -3931,7 +3947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="3:7">
       <c r="C58" s="4"/>
       <c r="D58" s="5"/>
       <c r="E58" s="4" t="s">
@@ -3944,7 +3960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="3:7">
       <c r="C59" s="4"/>
       <c r="D59" s="5"/>
       <c r="E59" s="4" t="s">
@@ -3957,7 +3973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="3:7">
       <c r="C60" s="4"/>
       <c r="D60" s="5"/>
       <c r="E60" s="4" t="s">
@@ -3970,7 +3986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="3:7">
       <c r="C61" s="4"/>
       <c r="D61" s="5"/>
       <c r="E61" s="4" t="s">
@@ -3983,7 +3999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="3:7">
       <c r="C62" s="4"/>
       <c r="D62" s="5"/>
       <c r="E62" s="4" t="s">
@@ -3996,7 +4012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="3:7">
       <c r="C63" s="4"/>
       <c r="D63" s="5"/>
       <c r="E63" s="4" t="s">
@@ -4009,7 +4025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="3:7">
       <c r="C64" s="4"/>
       <c r="D64" s="5"/>
       <c r="E64" s="4" t="s">
@@ -4022,7 +4038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:7">
       <c r="C65" s="4"/>
       <c r="D65" s="5"/>
       <c r="E65" s="4" t="s">
@@ -4035,7 +4051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="3:7">
       <c r="C66" s="4"/>
       <c r="D66" s="5"/>
       <c r="E66" s="4" t="s">

</xml_diff>